<commit_message>
Add searchable Projektakten workbook with filters
Replace the unusable pile of single-project files as the main entry with
Projektakten_Suche.xlsx (also as Projektakte.xlsx): AutoFilter on all
projects, dropdown Auswahl sheet, filterable Rechnungen/Forecast/Stunden.

Co-authored-by: fabsieb-boop <fabsieb-boop@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/workbook-split/projektakten/00_Projektakten_Uebersicht.xlsx
+++ b/docs/workbook-split/projektakten/00_Projektakten_Uebersicht.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Uebersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Uebersicht'!$A$4:$J$172</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,6 +36,18 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -48,7 +62,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -56,20 +70,40 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D0D7DE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D0D7DE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D0D7DE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D0D7DE"/>
+      </bottom>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -432,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I172"/>
+  <dimension ref="A1:J172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -460,51 +494,55 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Projekt-Nr.</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Leistung SAP</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Var. Kosten</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>DB4</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Buchungen</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Datei</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Suchtext</t>
         </is>
       </c>
     </row>
@@ -541,9 +579,14 @@
       <c r="H5" t="n">
         <v>49</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157208_Waggonverschrottung.xlsx</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>p4102157208 waggonverschrottung west abgeschlossen -46266.37</t>
         </is>
       </c>
     </row>
@@ -580,9 +623,14 @@
       <c r="H6" t="n">
         <v>2</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157411_ARGE_RB_Chemiepark_Krefeld.xlsx</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>p4102157411 arge rb chemiepark krefeld west aktiv 45582.42</t>
         </is>
       </c>
     </row>
@@ -619,9 +667,14 @@
       <c r="H7" t="n">
         <v>59</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157414_Krandemontage.xlsx</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>p4102157414 krandemontage west aktiv 135971.81</t>
         </is>
       </c>
     </row>
@@ -658,9 +711,14 @@
       <c r="H8" t="n">
         <v>46</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I8" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157420_ARGE_RB_GWA_SGA_4.xlsx</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>p4102157420 arge rb gwa+sga 4 west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -697,9 +755,14 @@
       <c r="H9" t="n">
         <v>40</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I9" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157429_Covestro_-_Rückbau_LEV_O13.xlsx</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>p4102157429 covestro - rückbau lev o13 west aktiv 59.31</t>
         </is>
       </c>
     </row>
@@ -736,9 +799,14 @@
       <c r="H10" t="n">
         <v>4</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I10" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157431_RB_drei_Sandfilter.xlsx</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>p4102157431 rb drei sandfilter west abgeschlossen -5683.12</t>
         </is>
       </c>
     </row>
@@ -775,9 +843,14 @@
       <c r="H11" t="n">
         <v>4</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I11" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157436_Sanierung_Kompensatoren.xlsx</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>p4102157436 sanierung kompensatoren west abgeschlossen 5236.57</t>
         </is>
       </c>
     </row>
@@ -814,9 +887,14 @@
       <c r="H12" t="n">
         <v>2</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I12" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157439_RB_Sperrmüllschereefeld.xlsx</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>p4102157439 rb sperrmüllschereefeld west abgeschlossen 37284</t>
         </is>
       </c>
     </row>
@@ -853,9 +931,14 @@
       <c r="H13" t="n">
         <v>6</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I13" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157440_tkse_RB_2025.xlsx</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>p4102157440 tkse rb 2025 west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -892,9 +975,14 @@
       <c r="H14" t="n">
         <v>81</v>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I14" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157442_RB_Leitstand_Flämmaschine.xlsx</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>p4102157442 rb leitstand flämmaschine west aktiv 48086.9</t>
         </is>
       </c>
     </row>
@@ -931,9 +1019,14 @@
       <c r="H15" t="n">
         <v>8</v>
       </c>
-      <c r="I15" t="inlineStr">
+      <c r="I15" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157443_Medice_Arzneim_RB_2_Tanks.xlsx</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>p4102157443 medice arzneim. rb 2 tanks west abgeschlossen 7269.84</t>
         </is>
       </c>
     </row>
@@ -970,9 +1063,14 @@
       <c r="H16" t="n">
         <v>8</v>
       </c>
-      <c r="I16" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157445_RB_2_Stahlwände_Lüra_Halle.xlsx</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>p4102157445 rb 2 stahlwände lüra halle west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -1009,9 +1107,14 @@
       <c r="H17" t="n">
         <v>2</v>
       </c>
-      <c r="I17" t="inlineStr">
+      <c r="I17" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157447_Hkm_Demontage_DN_500.xlsx</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>p4102157447 hkm demontage dn 500 west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -1048,9 +1151,14 @@
       <c r="H18" t="n">
         <v>141</v>
       </c>
-      <c r="I18" t="inlineStr">
+      <c r="I18" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157449_RB_Kessel_KW_Lausward.xlsx</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>p4102157449 rb kessel kw lausward west aktiv 248519.28</t>
         </is>
       </c>
     </row>
@@ -1087,9 +1195,14 @@
       <c r="H19" t="n">
         <v>10</v>
       </c>
-      <c r="I19" t="inlineStr">
+      <c r="I19" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157450_Verschr_Brennkammer_BA-301_Oxygen.xlsx</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>p4102157450 verschr. brennkammer ba-301 oxygen west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -1126,9 +1239,14 @@
       <c r="H20" t="n">
         <v>541</v>
       </c>
-      <c r="I20" t="inlineStr">
+      <c r="I20" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157451_Sanierung_Campus_Golzheim.xlsx</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>p4102157451 sanierung campus golzheim west aktiv 2069335.5</t>
         </is>
       </c>
     </row>
@@ -1165,9 +1283,14 @@
       <c r="H21" t="n">
         <v>2</v>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I21" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157452_RB_Cont_anlage_TKSE_Gelände.xlsx</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>p4102157452 rb cont.anlage tkse gelände west abgeschlossen -2847.73</t>
         </is>
       </c>
     </row>
@@ -1204,9 +1327,14 @@
       <c r="H22" t="n">
         <v>321</v>
       </c>
-      <c r="I22" t="inlineStr">
+      <c r="I22" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157453_Wbw_4_Hallenrückbau.xlsx</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>p4102157453 wbw 4 hallenrückbau west aktiv 1061843.93</t>
         </is>
       </c>
     </row>
@@ -1243,9 +1371,14 @@
       <c r="H23" t="n">
         <v>526</v>
       </c>
-      <c r="I23" t="inlineStr">
+      <c r="I23" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157455_Currenta_San_RB_G22_Los_1_2_Anm_fehlt.xlsx</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>p4102157455 currenta san.+rb g22 los 1+2 anm.fehlt west aktiv 2639009.53</t>
         </is>
       </c>
     </row>
@@ -1273,9 +1406,14 @@
       <c r="H24" t="n">
         <v>0</v>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I24" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157455-01_Los_1_Schadstoffsanierung.xlsx</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>p4102157455-01 los 1 schadstoffsanierung west aktiv</t>
         </is>
       </c>
     </row>
@@ -1303,9 +1441,14 @@
       <c r="H25" t="n">
         <v>0</v>
       </c>
-      <c r="I25" t="inlineStr">
+      <c r="I25" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157455-02_Los_2_Rückbau_und_Entsorgung.xlsx</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>p4102157455-02 los 2 rückbau und entsorgung west aktiv</t>
         </is>
       </c>
     </row>
@@ -1342,9 +1485,14 @@
       <c r="H26" t="n">
         <v>57</v>
       </c>
-      <c r="I26" t="inlineStr">
+      <c r="I26" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157456_RB_und_Entsorgung_Fundament_Schleifbank.xlsx</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>p4102157456 rb und entsorgung fundament schleifbank west aktiv 103280</t>
         </is>
       </c>
     </row>
@@ -1381,9 +1529,14 @@
       <c r="H27" t="n">
         <v>185</v>
       </c>
-      <c r="I27" t="inlineStr">
+      <c r="I27" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157457_tkse_RB_2026.xlsx</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>p4102157457 tkse rb 2026 west aktiv 273337.79</t>
         </is>
       </c>
     </row>
@@ -1420,9 +1573,14 @@
       <c r="H28" t="n">
         <v>44</v>
       </c>
-      <c r="I28" t="inlineStr">
+      <c r="I28" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157458_Kleinaufträge_Region_West_2026.xlsx</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>p4102157458 kleinaufträge region west 2026 west aktiv 27473.13</t>
         </is>
       </c>
     </row>
@@ -1459,9 +1617,14 @@
       <c r="H29" t="n">
         <v>28</v>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157459_RB_alte_Beizanlage.xlsx</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>p4102157459 rb alte beizanlage west aktiv 32538</t>
         </is>
       </c>
     </row>
@@ -1498,9 +1661,14 @@
       <c r="H30" t="n">
         <v>48</v>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I30" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157461_Brücke_D_1_Seitenteile.xlsx</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>p4102157461 brücke d 1 seitenteile west aktiv 37000</t>
         </is>
       </c>
     </row>
@@ -1537,9 +1705,14 @@
       <c r="H31" t="n">
         <v>42</v>
       </c>
-      <c r="I31" t="inlineStr">
+      <c r="I31" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157462_Waggonverschrottung_2026.xlsx</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>p4102157462 waggonverschrottung 2026 west aktiv 18107.39</t>
         </is>
       </c>
     </row>
@@ -1576,9 +1749,14 @@
       <c r="H32" t="n">
         <v>149</v>
       </c>
-      <c r="I32" t="inlineStr">
+      <c r="I32" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157463_RB_Maschinenhaus_Bl_B_C.xlsx</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>p4102157463 rb maschinenhaus bl. b+c west aktiv 758485.81</t>
         </is>
       </c>
     </row>
@@ -1615,9 +1793,14 @@
       <c r="H33" t="n">
         <v>22</v>
       </c>
-      <c r="I33" t="inlineStr">
+      <c r="I33" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157464_Asbest_Schadstoffsanierung_C_601.xlsx</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>p4102157464 asbest schadstoffsanierung c 601 west aktiv 23745</t>
         </is>
       </c>
     </row>
@@ -1654,9 +1837,14 @@
       <c r="H34" t="n">
         <v>15</v>
       </c>
-      <c r="I34" t="inlineStr">
+      <c r="I34" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157465_Reinigungsarbeiten_Block_B.xlsx</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>p4102157465 reinigungsarbeiten block b west aktiv 16000</t>
         </is>
       </c>
     </row>
@@ -1693,9 +1881,14 @@
       <c r="H35" t="n">
         <v>27</v>
       </c>
-      <c r="I35" t="inlineStr">
+      <c r="I35" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157466_Verschrottung_Anlagenteile.xlsx</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>p4102157466 verschrottung anlagenteile west aktiv 15250</t>
         </is>
       </c>
     </row>
@@ -1732,9 +1925,14 @@
       <c r="H36" t="n">
         <v>10</v>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I36" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157467_Plakoma_-_Dem_Roheisenfähren.xlsx</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>p4102157467 plakoma - dem. roheisenfähren west aktiv 220000</t>
         </is>
       </c>
     </row>
@@ -1771,9 +1969,14 @@
       <c r="H37" t="n">
         <v>4</v>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I37" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157468_Verschr_Kondensattank_Kokerei_Schwelger.xlsx</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>p4102157468 verschr. kondensattank kokerei schwelger west aktiv -10600</t>
         </is>
       </c>
     </row>
@@ -1810,9 +2013,14 @@
       <c r="H38" t="n">
         <v>5</v>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I38" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157469_Anmeldung_fehlt.xlsx</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>p4102157469 anmeldung fehlt west aktiv</t>
         </is>
       </c>
     </row>
@@ -1849,9 +2057,14 @@
       <c r="H39" t="n">
         <v>0</v>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I39" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157470_Sägetechn_Demontage_Mischgasleitung.xlsx</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>p4102157470 sägetechn demontage mischgasleitung west aktiv</t>
         </is>
       </c>
     </row>
@@ -1888,9 +2101,14 @@
       <c r="H40" t="n">
         <v>0</v>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102157472_Kaltwindleitung_SMB.xlsx</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>p4102157472 kaltwindleitung smb west aktiv</t>
         </is>
       </c>
     </row>
@@ -1927,9 +2145,14 @@
       <c r="H41" t="n">
         <v>48</v>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307304_HKW_Süd.xlsx</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>p4102307304 hkw süd süd-west aktiv 124.95</t>
         </is>
       </c>
     </row>
@@ -1966,9 +2189,14 @@
       <c r="H42" t="n">
         <v>4</v>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307306_RB_Halle_Karlsruhe.xlsx</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>p4102307306 rb halle karlsruhe süd-west aktiv -35814.88</t>
         </is>
       </c>
     </row>
@@ -2005,9 +2233,14 @@
       <c r="H43" t="n">
         <v>2</v>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307411_BASF_G_521.xlsx</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>p4102307411 basf g 521 süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -2044,9 +2277,14 @@
       <c r="H44" t="n">
         <v>2</v>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307416_BASF_O_405_Ammoniak.xlsx</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>p4102307416 basf o 405 ammoniak süd-west abgeschlossen -25780.46</t>
         </is>
       </c>
     </row>
@@ -2083,9 +2321,14 @@
       <c r="H45" t="n">
         <v>18</v>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307422_BASF_M_950.xlsx</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>p4102307422 basf m 950 süd-west abgeschlossen -8740.15</t>
         </is>
       </c>
     </row>
@@ -2122,9 +2365,14 @@
       <c r="H46" t="n">
         <v>12</v>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307423_BASF_F_712.xlsx</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>p4102307423 basf f 712 süd-west abgeschlossen 29755.02</t>
         </is>
       </c>
     </row>
@@ -2161,9 +2409,14 @@
       <c r="H47" t="n">
         <v>6</v>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307424_BASF_P_703.xlsx</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>p4102307424 basf p 703 süd-west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -2200,9 +2453,14 @@
       <c r="H48" t="n">
         <v>20</v>
       </c>
-      <c r="I48" t="inlineStr">
+      <c r="I48" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307426_BASF_Z_300.xlsx</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>p4102307426 basf z 300 süd-west abgeschlossen 40236.26</t>
         </is>
       </c>
     </row>
@@ -2239,9 +2497,14 @@
       <c r="H49" t="n">
         <v>62</v>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I49" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307427_BASF_N_720.xlsx</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>p4102307427 basf n 720 süd-west aktiv 40570.44</t>
         </is>
       </c>
     </row>
@@ -2278,9 +2541,14 @@
       <c r="H50" t="n">
         <v>82</v>
       </c>
-      <c r="I50" t="inlineStr">
+      <c r="I50" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307428_BASF_O_405.xlsx</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>p4102307428 basf o 405 süd-west aktiv 149536.25</t>
         </is>
       </c>
     </row>
@@ -2317,9 +2585,14 @@
       <c r="H51" t="n">
         <v>47</v>
       </c>
-      <c r="I51" t="inlineStr">
+      <c r="I51" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307429_BASF_C_509.xlsx</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>p4102307429 basf c 509 süd-west aktiv 33120.57</t>
         </is>
       </c>
     </row>
@@ -2356,9 +2629,14 @@
       <c r="H52" t="n">
         <v>31</v>
       </c>
-      <c r="I52" t="inlineStr">
+      <c r="I52" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307430_BASF_E_701.xlsx</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>p4102307430 basf e 701 süd-west aktiv 41935.11</t>
         </is>
       </c>
     </row>
@@ -2395,9 +2673,14 @@
       <c r="H53" t="n">
         <v>4</v>
       </c>
-      <c r="I53" t="inlineStr">
+      <c r="I53" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307431_HNVG_Bauph_II_Gaswerk.xlsx</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>p4102307431 hnvg bauph. ii gaswerk süd-west abgeschlossen 14290.34</t>
         </is>
       </c>
     </row>
@@ -2434,9 +2717,14 @@
       <c r="H54" t="n">
         <v>22</v>
       </c>
-      <c r="I54" t="inlineStr">
+      <c r="I54" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307432_HNVG_-_Bauph_III_Gaswerk.xlsx</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>p4102307432 hnvg - bauph. iii gaswerk süd-west abgeschlossen 45525.16</t>
         </is>
       </c>
     </row>
@@ -2473,9 +2761,14 @@
       <c r="H55" t="n">
         <v>381</v>
       </c>
-      <c r="I55" t="inlineStr">
+      <c r="I55" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307433_BASF_U_505_Blauer_Block.xlsx</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>p4102307433 basf u 505 blauer block süd-west aktiv 845407</t>
         </is>
       </c>
     </row>
@@ -2512,9 +2805,14 @@
       <c r="H56" t="n">
         <v>36</v>
       </c>
-      <c r="I56" t="inlineStr">
+      <c r="I56" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307434_BASF_S_304.xlsx</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>p4102307434 basf s 304 süd-west abgeschlossen 13933.04</t>
         </is>
       </c>
     </row>
@@ -2551,9 +2849,14 @@
       <c r="H57" t="n">
         <v>101</v>
       </c>
-      <c r="I57" t="inlineStr">
+      <c r="I57" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307435_ENBW_-_KW_Walheim.xlsx</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>p4102307435 enbw - kw walheim süd-west abgeschlossen 72370.01</t>
         </is>
       </c>
     </row>
@@ -2590,9 +2893,14 @@
       <c r="H58" t="n">
         <v>77</v>
       </c>
-      <c r="I58" t="inlineStr">
+      <c r="I58" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307436_BASF_O_914_-_O_915.xlsx</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>p4102307436 basf o 914 - o 915 süd-west aktiv 57545.38</t>
         </is>
       </c>
     </row>
@@ -2629,9 +2937,14 @@
       <c r="H59" t="n">
         <v>30</v>
       </c>
-      <c r="I59" t="inlineStr">
+      <c r="I59" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307437_ENBW_-_KW_Walheim_Permutit-Anlage.xlsx</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>p4102307437 enbw - kw walheim, permutit-anlage süd-west abgeschlossen 49.86</t>
         </is>
       </c>
     </row>
@@ -2668,9 +2981,14 @@
       <c r="H60" t="n">
         <v>49</v>
       </c>
-      <c r="I60" t="inlineStr">
+      <c r="I60" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307438_Netze_BW-_UW_Bruchsal.xlsx</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>p4102307438 netze bw- uw bruchsal süd-west aktiv 62025.81</t>
         </is>
       </c>
     </row>
@@ -2707,9 +3025,14 @@
       <c r="H61" t="n">
         <v>97</v>
       </c>
-      <c r="I61" t="inlineStr">
+      <c r="I61" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307439_BASF_U_405_Teil_1.xlsx</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>p4102307439 basf u 405 teil 1 süd-west aktiv 73270.25</t>
         </is>
       </c>
     </row>
@@ -2746,9 +3069,14 @@
       <c r="H62" t="n">
         <v>161</v>
       </c>
-      <c r="I62" t="inlineStr">
+      <c r="I62" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307440_BASF_L_605.xlsx</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>p4102307440 basf  l 605 süd-west aktiv 249898.21</t>
         </is>
       </c>
     </row>
@@ -2785,9 +3113,14 @@
       <c r="H63" t="n">
         <v>78</v>
       </c>
-      <c r="I63" t="inlineStr">
+      <c r="I63" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307441_BASF_E_301.xlsx</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>p4102307441 basf  e 301 süd-west abgeschlossen 12625.47</t>
         </is>
       </c>
     </row>
@@ -2824,9 +3157,14 @@
       <c r="H64" t="n">
         <v>41</v>
       </c>
-      <c r="I64" t="inlineStr">
+      <c r="I64" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307442_Leingarten_Schwimmhalle_1.xlsx</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>p4102307442 leingarten schwimmhalle 1 süd-west aktiv 84738.88</t>
         </is>
       </c>
     </row>
@@ -2863,9 +3201,14 @@
       <c r="H65" t="n">
         <v>7</v>
       </c>
-      <c r="I65" t="inlineStr">
+      <c r="I65" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307443_Leingarten_Schwimmhalle_2.xlsx</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>p4102307443 leingarten schwimmhalle 2 süd-west aktiv 121773.65</t>
         </is>
       </c>
     </row>
@@ -2902,9 +3245,14 @@
       <c r="H66" t="n">
         <v>103</v>
       </c>
-      <c r="I66" t="inlineStr">
+      <c r="I66" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307444_BASF_N_416-O_405.xlsx</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>p4102307444 basf  n 416-o 405 süd-west aktiv 53164.67</t>
         </is>
       </c>
     </row>
@@ -2941,9 +3289,14 @@
       <c r="H67" t="n">
         <v>16</v>
       </c>
-      <c r="I67" t="inlineStr">
+      <c r="I67" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307447_BASF_C_317.xlsx</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>p4102307447 basf c 317 süd-west aktiv 32751.02</t>
         </is>
       </c>
     </row>
@@ -2980,9 +3333,14 @@
       <c r="H68" t="n">
         <v>11</v>
       </c>
-      <c r="I68" t="inlineStr">
+      <c r="I68" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307448_Kopf_SynGas_-_Klärschlammvergasung.xlsx</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>p4102307448 kopf syngas - klärschlammvergasung süd-west aktiv 9829.8</t>
         </is>
       </c>
     </row>
@@ -3019,9 +3377,14 @@
       <c r="H69" t="n">
         <v>13</v>
       </c>
-      <c r="I69" t="inlineStr">
+      <c r="I69" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307449_BASF_S_607.xlsx</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>p4102307449 basf s 607 süd-west aktiv 20000</t>
         </is>
       </c>
     </row>
@@ -3058,9 +3421,14 @@
       <c r="H70" t="n">
         <v>0</v>
       </c>
-      <c r="I70" t="inlineStr">
+      <c r="I70" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307450_Z500-4_Helion.xlsx</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>p4102307450 z500-4 helion süd-west aktiv 132500</t>
         </is>
       </c>
     </row>
@@ -3088,9 +3456,14 @@
       <c r="H71" t="n">
         <v>0</v>
       </c>
-      <c r="I71" t="inlineStr">
+      <c r="I71" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102307455_BASF_Z500.xlsx</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>p4102307455 basf z500 süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -3127,9 +3500,14 @@
       <c r="H72" t="n">
         <v>2</v>
       </c>
-      <c r="I72" t="inlineStr">
+      <c r="I72" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102309044_RB_BASF_2022.xlsx</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>p4102309044 rb basf 2022 süd-west aktiv -6447.83</t>
         </is>
       </c>
     </row>
@@ -3166,9 +3544,14 @@
       <c r="H73" t="n">
         <v>129</v>
       </c>
-      <c r="I73" t="inlineStr">
+      <c r="I73" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102309045_BASF_Sonstige_Kleinmaßnahmen.xlsx</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>p4102309045 basf sonstige kleinmaßnahmen süd-west aktiv 131609.09</t>
         </is>
       </c>
     </row>
@@ -3205,9 +3588,14 @@
       <c r="H74" t="n">
         <v>20</v>
       </c>
-      <c r="I74" t="inlineStr">
+      <c r="I74" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102309046_Sonstige_Kleinmaßnahmen.xlsx</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>p4102309046 sonstige kleinmaßnahmen süd-west aktiv 24410.59</t>
         </is>
       </c>
     </row>
@@ -3244,9 +3632,14 @@
       <c r="H75" t="n">
         <v>26</v>
       </c>
-      <c r="I75" t="inlineStr">
+      <c r="I75" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102602023_nachlaufende_Kosten.xlsx</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>p4102602023 nachlaufende kosten ost aktiv</t>
         </is>
       </c>
     </row>
@@ -3283,9 +3676,14 @@
       <c r="H76" t="n">
         <v>15</v>
       </c>
-      <c r="I76" t="inlineStr">
+      <c r="I76" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102604612_Recyclingplatz_Boxberg.xlsx</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>p4102604612 recyclingplatz boxberg ost aktiv 1055.73</t>
         </is>
       </c>
     </row>
@@ -3322,9 +3720,14 @@
       <c r="H77" t="n">
         <v>202</v>
       </c>
-      <c r="I77" t="inlineStr">
+      <c r="I77" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102607989_Kleinaufträge.xlsx</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>p4102607989 kleinaufträge ost aktiv 98017.2</t>
         </is>
       </c>
     </row>
@@ -3361,9 +3764,14 @@
       <c r="H78" t="n">
         <v>7</v>
       </c>
-      <c r="I78" t="inlineStr">
+      <c r="I78" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608224_RB_Turbinen_Hirschfelde.xlsx</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>p4102608224 rb turbinen hirschfelde ost aktiv 1969.8</t>
         </is>
       </c>
     </row>
@@ -3400,9 +3808,14 @@
       <c r="H79" t="n">
         <v>2</v>
       </c>
-      <c r="I79" t="inlineStr">
+      <c r="I79" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608226_RB_Kohlebunker_Lübbenau.xlsx</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>p4102608226 rb kohlebunker lübbenau ost aktiv</t>
         </is>
       </c>
     </row>
@@ -3439,9 +3852,14 @@
       <c r="H80" t="n">
         <v>2</v>
       </c>
-      <c r="I80" t="inlineStr">
+      <c r="I80" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608232_Seilbaggerarbeiten_Platz_der_Republik.xlsx</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>p4102608232 seilbaggerarbeiten platz der republik ost abgeschlossen 6059.53</t>
         </is>
       </c>
     </row>
@@ -3478,9 +3896,14 @@
       <c r="H81" t="n">
         <v>520</v>
       </c>
-      <c r="I81" t="inlineStr">
+      <c r="I81" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608246_RB_Kohlebunker_Brücke_Lübbenau.xlsx</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>p4102608246 rb kohlebunker/brücke lübbenau ost aktiv 832368.22</t>
         </is>
       </c>
     </row>
@@ -3517,9 +3940,14 @@
       <c r="H82" t="n">
         <v>4</v>
       </c>
-      <c r="I82" t="inlineStr">
+      <c r="I82" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608258_BTU_Dachsanierung_Halle_3b.xlsx</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>p4102608258 btu dachsanierung halle 3b ost abgeschlossen 81006.27</t>
         </is>
       </c>
     </row>
@@ -3556,9 +3984,14 @@
       <c r="H83" t="n">
         <v>57</v>
       </c>
-      <c r="I83" t="inlineStr">
+      <c r="I83" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608260_RB_Floorflexplatten_Berlin.xlsx</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>p4102608260 rb floorflexplatten berlin ost aktiv 16839.08</t>
         </is>
       </c>
     </row>
@@ -3595,9 +4028,14 @@
       <c r="H84" t="n">
         <v>296</v>
       </c>
-      <c r="I84" t="inlineStr">
+      <c r="I84" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608263_RB_Föderbrücke_AFB_60.xlsx</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>p4102608263 rb föderbrücke afb 60 ost aktiv 2991108.78</t>
         </is>
       </c>
     </row>
@@ -3634,9 +4072,14 @@
       <c r="H85" t="n">
         <v>8</v>
       </c>
-      <c r="I85" t="inlineStr">
+      <c r="I85" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608264_Mastrückbau_Mainflingen.xlsx</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>p4102608264 mastrückbau mainflingen ost abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -3673,9 +4116,14 @@
       <c r="H86" t="n">
         <v>20</v>
       </c>
-      <c r="I86" t="inlineStr">
+      <c r="I86" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608265_RB_Gebäude_Grüneberg.xlsx</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>p4102608265 rb gebäude grüneberg ost abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -3712,9 +4160,14 @@
       <c r="H87" t="n">
         <v>10</v>
       </c>
-      <c r="I87" t="inlineStr">
+      <c r="I87" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608266_RB_Kurmark-_Kaserne_Storkow.xlsx</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>p4102608266 rb kurmark- kaserne storkow ost abgeschlossen -591.81</t>
         </is>
       </c>
     </row>
@@ -3751,9 +4204,14 @@
       <c r="H88" t="n">
         <v>39</v>
       </c>
-      <c r="I88" t="inlineStr">
+      <c r="I88" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608267_Sprengarbeiten_FLJS.xlsx</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>p4102608267 sprengarbeiten fljs ost abgeschlossen 28224.24</t>
         </is>
       </c>
     </row>
@@ -3790,9 +4248,14 @@
       <c r="H89" t="n">
         <v>27</v>
       </c>
-      <c r="I89" t="inlineStr">
+      <c r="I89" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608268_Gutenbergstrasse_Potsdam.xlsx</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>p4102608268 gutenbergstrasse potsdam ost abgeschlossen 5542.71</t>
         </is>
       </c>
     </row>
@@ -3829,9 +4292,14 @@
       <c r="H90" t="n">
         <v>93</v>
       </c>
-      <c r="I90" t="inlineStr">
+      <c r="I90" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608270_Baggergestellung_LH_956_Jänschwalde.xlsx</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>p4102608270 baggergestellung lh 956 jänschwalde ost aktiv 99403.64</t>
         </is>
       </c>
     </row>
@@ -3868,9 +4336,14 @@
       <c r="H91" t="n">
         <v>64</v>
       </c>
-      <c r="I91" t="inlineStr">
+      <c r="I91" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608271_Seilbagger_Tagebau_Jänschwalde.xlsx</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>p4102608271 seilbagger tagebau jänschwalde ost aktiv 156757.06</t>
         </is>
       </c>
     </row>
@@ -3907,9 +4380,14 @@
       <c r="H92" t="n">
         <v>19</v>
       </c>
-      <c r="I92" t="inlineStr">
+      <c r="I92" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608275_An_der_Spreewaldbahn_lübben.xlsx</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>p4102608275 an der spreewaldbahn lübben ost aktiv</t>
         </is>
       </c>
     </row>
@@ -3946,9 +4424,14 @@
       <c r="H93" t="n">
         <v>0</v>
       </c>
-      <c r="I93" t="inlineStr">
+      <c r="I93" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102608277_Siebarbeiten_KMK_Storkow.xlsx</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>p4102608277 siebarbeiten kmk storkow ost aktiv 9367.07</t>
         </is>
       </c>
     </row>
@@ -3985,9 +4468,14 @@
       <c r="H94" t="n">
         <v>4</v>
       </c>
-      <c r="I94" t="inlineStr">
+      <c r="I94" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102652023_Nachlaufende_Kosten.xlsx</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>p4102652023 nachlaufende kosten berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -4024,9 +4512,14 @@
       <c r="H95" t="n">
         <v>8</v>
       </c>
-      <c r="I95" t="inlineStr">
+      <c r="I95" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102657982_Kleinaufträge.xlsx</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>p4102657982 kleinaufträge berlin aktiv 8250</t>
         </is>
       </c>
     </row>
@@ -4063,9 +4556,14 @@
       <c r="H96" t="n">
         <v>9</v>
       </c>
-      <c r="I96" t="inlineStr">
+      <c r="I96" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658225_B1_Brandenburg_Potsdamer_Straße.xlsx</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>p4102658225 b1 brandenburg potsdamer straße berlin aktiv -122785.46</t>
         </is>
       </c>
     </row>
@@ -4102,9 +4600,14 @@
       <c r="H97" t="n">
         <v>6</v>
       </c>
-      <c r="I97" t="inlineStr">
+      <c r="I97" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658228_ENB_EÜ_Wollankstraße.xlsx</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>p4102658228 enb eü wollankstraße berlin aktiv 475.29</t>
         </is>
       </c>
     </row>
@@ -4141,9 +4644,14 @@
       <c r="H98" t="n">
         <v>319</v>
       </c>
-      <c r="I98" t="inlineStr">
+      <c r="I98" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658229_Markgrafenbrücke_Berlin.xlsx</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>p4102658229 markgrafenbrücke berlin berlin aktiv 527418.28</t>
         </is>
       </c>
     </row>
@@ -4180,9 +4688,14 @@
       <c r="H99" t="n">
         <v>4</v>
       </c>
-      <c r="I99" t="inlineStr">
+      <c r="I99" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658235_ENB_Neue_Fahlenbergbrücke.xlsx</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>p4102658235 enb neue fahlenbergbrücke berlin abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -4219,9 +4732,14 @@
       <c r="H100" t="n">
         <v>24</v>
       </c>
-      <c r="I100" t="inlineStr">
+      <c r="I100" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658250_Parkallee_Velten_Brücke_Stichkanal.xlsx</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>p4102658250 parkallee velten, brücke stichkanal berlin abgeschlossen -39809.7</t>
         </is>
       </c>
     </row>
@@ -4258,9 +4776,14 @@
       <c r="H101" t="n">
         <v>7</v>
       </c>
-      <c r="I101" t="inlineStr">
+      <c r="I101" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658254_EÜ_Langendreerstraße_Bochum.xlsx</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>p4102658254 eü langendreerstraße bochum berlin abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -4297,9 +4820,14 @@
       <c r="H102" t="n">
         <v>200</v>
       </c>
-      <c r="I102" t="inlineStr">
+      <c r="I102" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658256_Schleuse_Wolfswinkel.xlsx</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>p4102658256 schleuse wolfswinkel berlin aktiv 231904.97</t>
         </is>
       </c>
     </row>
@@ -4336,9 +4864,14 @@
       <c r="H103" t="n">
         <v>4</v>
       </c>
-      <c r="I103" t="inlineStr">
+      <c r="I103" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658257_Brücke_An_der_Wuhlheide_-_Notunterstützu.xlsx</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>p4102658257 brücke an der wuhlheide - notunterstützu berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -4375,9 +4908,14 @@
       <c r="H104" t="n">
         <v>9</v>
       </c>
-      <c r="I104" t="inlineStr">
+      <c r="I104" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658259_ENB_Eisenbahnbrücke_Güsen.xlsx</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>p4102658259 enb eisenbahnbrücke güsen berlin aktiv 52101.99</t>
         </is>
       </c>
     </row>
@@ -4414,9 +4952,14 @@
       <c r="H105" t="n">
         <v>57</v>
       </c>
-      <c r="I105" t="inlineStr">
+      <c r="I105" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658269_B102_OD_Jüterbog_Alte_Nuthe.xlsx</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>p4102658269 b102 od jüterbog alte nuthe berlin abgeschlossen 16030.23</t>
         </is>
       </c>
     </row>
@@ -4453,9 +4996,14 @@
       <c r="H106" t="n">
         <v>83</v>
       </c>
-      <c r="I106" t="inlineStr">
+      <c r="I106" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658272_Beräumung_Herzberger_Straße.xlsx</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>p4102658272 beräumung herzberger straße berlin aktiv 36922.66</t>
         </is>
       </c>
     </row>
@@ -4492,9 +5040,14 @@
       <c r="H107" t="n">
         <v>100</v>
       </c>
-      <c r="I107" t="inlineStr">
+      <c r="I107" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658276_EÜ_Braunsbedra.xlsx</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>p4102658276 eü braunsbedra berlin aktiv 98022.87</t>
         </is>
       </c>
     </row>
@@ -4522,9 +5075,14 @@
       <c r="H108" t="n">
         <v>0</v>
       </c>
-      <c r="I108" t="inlineStr">
+      <c r="I108" s="5" t="inlineStr">
         <is>
           <t>Projekt_P4102658277_Brücke_Uechtingstraße_Gelsenkirchen.xlsx</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>p4102658277 brücke uechtingstraße, gelsenkirchen berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -4552,9 +5110,14 @@
       <c r="H109" t="n">
         <v>599</v>
       </c>
-      <c r="I109" t="inlineStr">
+      <c r="I109" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154411_Vetrieb_Region_West.xlsx</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>w4102154411 vetrieb region west west aktiv</t>
         </is>
       </c>
     </row>
@@ -4582,9 +5145,14 @@
       <c r="H110" t="n">
         <v>9</v>
       </c>
-      <c r="I110" t="inlineStr">
+      <c r="I110" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154501_Gehalt_BL_Region_West.xlsx</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>w4102154501 gehalt bl region west west aktiv</t>
         </is>
       </c>
     </row>
@@ -4612,9 +5180,14 @@
       <c r="H111" t="n">
         <v>155</v>
       </c>
-      <c r="I111" t="inlineStr">
+      <c r="I111" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154611_Werkstatt_Region_West.xlsx</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>w4102154611 werkstatt region west west aktiv</t>
         </is>
       </c>
     </row>
@@ -4642,9 +5215,14 @@
       <c r="H112" t="n">
         <v>9</v>
       </c>
-      <c r="I112" t="inlineStr">
+      <c r="I112" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154953_CB-AA_140_Hr_Kraft.xlsx</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>w4102154953 cb-aa 140 hr. kraft west aktiv</t>
         </is>
       </c>
     </row>
@@ -4672,9 +5250,14 @@
       <c r="H113" t="n">
         <v>55</v>
       </c>
-      <c r="I113" t="inlineStr">
+      <c r="I113" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154961_DO-AW_251_Ludwigs.xlsx</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>w4102154961 do-aw 251 ludwigs west aktiv</t>
         </is>
       </c>
     </row>
@@ -4702,9 +5285,14 @@
       <c r="H114" t="n">
         <v>36</v>
       </c>
-      <c r="I114" t="inlineStr">
+      <c r="I114" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154964_PKW_Schalk_CB_-_TV_93.xlsx</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>w4102154964 pkw schalk cb - tv 93 west aktiv</t>
         </is>
       </c>
     </row>
@@ -4732,9 +5320,14 @@
       <c r="H115" t="n">
         <v>19</v>
       </c>
-      <c r="I115" t="inlineStr">
+      <c r="I115" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154966_PKW_Kilinc.xlsx</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>w4102154966 pkw kilinc west aktiv</t>
         </is>
       </c>
     </row>
@@ -4762,9 +5355,14 @@
       <c r="H116" t="n">
         <v>38</v>
       </c>
-      <c r="I116" t="inlineStr">
+      <c r="I116" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154967_CB_-_VT_585_Hr_Büskens.xlsx</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>w4102154967 cb - vt 585  hr. büskens west aktiv</t>
         </is>
       </c>
     </row>
@@ -4792,9 +5390,14 @@
       <c r="H117" t="n">
         <v>1</v>
       </c>
-      <c r="I117" t="inlineStr">
+      <c r="I117" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102154968_PKW_Hr_Lanzar_Tore.xlsx</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>w4102154968 pkw hr. lanzar tore west aktiv</t>
         </is>
       </c>
     </row>
@@ -4822,9 +5425,14 @@
       <c r="H118" t="n">
         <v>2</v>
       </c>
-      <c r="I118" t="inlineStr">
+      <c r="I118" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102157414_Krandemontage.xlsx</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>w4102157414 krandemontage west aktiv</t>
         </is>
       </c>
     </row>
@@ -4852,9 +5460,14 @@
       <c r="H119" t="n">
         <v>459</v>
       </c>
-      <c r="I119" t="inlineStr">
+      <c r="I119" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304411_Vetrieb_Region_Sued-West.xlsx</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>w4102304411 vetrieb region sued-west süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -4882,9 +5495,14 @@
       <c r="H120" t="n">
         <v>32</v>
       </c>
-      <c r="I120" t="inlineStr">
+      <c r="I120" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304412_Fremdfirmenstuetzupunkt.xlsx</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>w4102304412 fremdfirmenstuetzupunkt süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -4912,9 +5530,14 @@
       <c r="H121" t="n">
         <v>212</v>
       </c>
-      <c r="I121" t="inlineStr">
+      <c r="I121" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304611_Lager_Region_Sued-West.xlsx</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>w4102304611 lager region sued-west süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -4942,9 +5565,14 @@
       <c r="H122" t="n">
         <v>39</v>
       </c>
-      <c r="I122" t="inlineStr">
+      <c r="I122" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304943_CB_-_TV_90_Hr_Flamme.xlsx</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>w4102304943 cb - tv 90 hr. flamme süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -4972,9 +5600,14 @@
       <c r="H123" t="n">
         <v>29</v>
       </c>
-      <c r="I123" t="inlineStr">
+      <c r="I123" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304946_CB-AA_552_Sesjunin.xlsx</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>w4102304946 cb-aa 552 sesjunin süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5002,9 +5635,14 @@
       <c r="H124" t="n">
         <v>8</v>
       </c>
-      <c r="I124" t="inlineStr">
+      <c r="I124" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304947_CB-AB_644_Passat_Herr_Yavuz.xlsx</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>w4102304947 cb-ab 644 passat herr yavuz süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5032,9 +5670,14 @@
       <c r="H125" t="n">
         <v>0</v>
       </c>
-      <c r="I125" t="inlineStr">
+      <c r="I125" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304948_AFB21202600801-0000000037.xlsx</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>w4102304948 afb21202600801-0000000037 süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5062,9 +5705,14 @@
       <c r="H126" t="n">
         <v>0</v>
       </c>
-      <c r="I126" t="inlineStr">
+      <c r="I126" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102304949_Service_CB-AA_552.xlsx</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>w4102304949 service cb-aa 552 süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5092,9 +5740,14 @@
       <c r="H127" t="n">
         <v>26</v>
       </c>
-      <c r="I127" t="inlineStr">
+      <c r="I127" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102307366_UW_Niederbühl.xlsx</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>w4102307366 uw niederbühl süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5122,9 +5775,14 @@
       <c r="H128" t="n">
         <v>1</v>
       </c>
-      <c r="I128" t="inlineStr">
+      <c r="I128" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102307411_BASF_-_G_521.xlsx</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>w4102307411 basf - g 521 süd-west abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -5152,9 +5810,14 @@
       <c r="H129" t="n">
         <v>0</v>
       </c>
-      <c r="I129" t="inlineStr">
+      <c r="I129" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102309045_Kleinmaßnahmen_BASF_2022.xlsx</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>w4102309045 kleinmaßnahmen basf 2022 süd-west aktiv</t>
         </is>
       </c>
     </row>
@@ -5182,9 +5845,14 @@
       <c r="H130" t="n">
         <v>6</v>
       </c>
-      <c r="I130" t="inlineStr">
+      <c r="I130" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504101_Kaufm_Geschäftsfüh.xlsx</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>w4102504101 kaufm. geschäftsfüh. verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5212,9 +5880,14 @@
       <c r="H131" t="n">
         <v>1</v>
       </c>
-      <c r="I131" t="inlineStr">
+      <c r="I131" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504102_Techn_Geschäftsfüh.xlsx</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>w4102504102 techn. geschäftsfüh. verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5242,9 +5915,14 @@
       <c r="H132" t="n">
         <v>10</v>
       </c>
-      <c r="I132" t="inlineStr">
+      <c r="I132" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504104_Dienstleistungsverrechn.xlsx</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>w4102504104 dienstleistungsverrechn. verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5272,9 +5950,14 @@
       <c r="H133" t="n">
         <v>68</v>
       </c>
-      <c r="I133" t="inlineStr">
+      <c r="I133" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504106_Geschäftsfüh.xlsx</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>w4102504106 geschäftsfüh. verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5302,9 +5985,14 @@
       <c r="H134" t="n">
         <v>17</v>
       </c>
-      <c r="I134" t="inlineStr">
+      <c r="I134" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504107_Geschäftsfüh_Hr_Kay.xlsx</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>w4102504107 geschäftsfüh. hr kay verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5332,9 +6020,14 @@
       <c r="H135" t="n">
         <v>44</v>
       </c>
-      <c r="I135" t="inlineStr">
+      <c r="I135" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504108_Geschäftsführer_Hr_Kenski.xlsx</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>w4102504108 geschäftsführer hr. kenski verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5362,9 +6055,14 @@
       <c r="H136" t="n">
         <v>36</v>
       </c>
-      <c r="I136" t="inlineStr">
+      <c r="I136" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504109_Geschäftsführerin_Frau_Langosch.xlsx</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>w4102504109 geschäftsführerin frau langosch verwaltung abgeschlossen</t>
         </is>
       </c>
     </row>
@@ -5392,9 +6090,14 @@
       <c r="H137" t="n">
         <v>10</v>
       </c>
-      <c r="I137" t="inlineStr">
+      <c r="I137" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504211_Rechnungsw_Finanzen.xlsx</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>w4102504211 rechnungsw./finanzen verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5422,9 +6125,14 @@
       <c r="H138" t="n">
         <v>24</v>
       </c>
-      <c r="I138" t="inlineStr">
+      <c r="I138" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504221_Übriges_Personal.xlsx</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>w4102504221 übriges personal verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5452,9 +6160,14 @@
       <c r="H139" t="n">
         <v>448</v>
       </c>
-      <c r="I139" t="inlineStr">
+      <c r="I139" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504222_Sonstige_Sachkosten.xlsx</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>w4102504222 sonstige sachkosten verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5482,9 +6195,14 @@
       <c r="H140" t="n">
         <v>119</v>
       </c>
-      <c r="I140" t="inlineStr">
+      <c r="I140" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504262_Zentrale_EDV.xlsx</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>w4102504262 zentrale edv verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5512,9 +6230,14 @@
       <c r="H141" t="n">
         <v>23</v>
       </c>
-      <c r="I141" t="inlineStr">
+      <c r="I141" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504941_Betriebsrat.xlsx</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>w4102504941 betriebsrat verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5542,9 +6265,14 @@
       <c r="H142" t="n">
         <v>28</v>
       </c>
-      <c r="I142" t="inlineStr">
+      <c r="I142" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504951_Steuern.xlsx</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>w4102504951 steuern verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5572,9 +6300,14 @@
       <c r="H143" t="n">
         <v>7</v>
       </c>
-      <c r="I143" t="inlineStr">
+      <c r="I143" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504967_CB-VT_476_Krull.xlsx</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>w4102504967 cb-vt 476 krull verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5602,9 +6335,14 @@
       <c r="H144" t="n">
         <v>25</v>
       </c>
-      <c r="I144" t="inlineStr">
+      <c r="I144" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504971_CB-CR_107_Werban.xlsx</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>w4102504971 cb-cr 107 werban verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5632,9 +6370,14 @@
       <c r="H145" t="n">
         <v>52</v>
       </c>
-      <c r="I145" t="inlineStr">
+      <c r="I145" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504973_CB-_TV_300E_Hr_Kemper_Mercedes.xlsx</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>w4102504973 cb- tv 300e hr. kemper mercedes verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5662,9 +6405,14 @@
       <c r="H146" t="n">
         <v>41</v>
       </c>
-      <c r="I146" t="inlineStr">
+      <c r="I146" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504974_CB-TV_55E_Volvo_Herr_Kay.xlsx</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>w4102504974 cb-tv 55e volvo herr kay verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5692,9 +6440,14 @@
       <c r="H147" t="n">
         <v>16</v>
       </c>
-      <c r="I147" t="inlineStr">
+      <c r="I147" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504975_PKW_Frau_Noack.xlsx</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>w4102504975 pkw frau noack verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5722,9 +6475,14 @@
       <c r="H148" t="n">
         <v>19</v>
       </c>
-      <c r="I148" t="inlineStr">
+      <c r="I148" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504976_CB-TV_104_Skoda_Superb_-_Herr_Kenski.xlsx</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>w4102504976 cb-tv 104 skoda superb - herr kenski verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5752,9 +6510,14 @@
       <c r="H149" t="n">
         <v>0</v>
       </c>
-      <c r="I149" t="inlineStr">
+      <c r="I149" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504977_PKW_Herr_Siebert.xlsx</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>w4102504977 pkw herr siebert verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5782,9 +6545,14 @@
       <c r="H150" t="n">
         <v>0</v>
       </c>
-      <c r="I150" t="inlineStr">
+      <c r="I150" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102504978_PKW_Frau_Mattiza.xlsx</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>w4102504978 pkw frau mattiza verwaltung aktiv</t>
         </is>
       </c>
     </row>
@@ -5812,9 +6580,14 @@
       <c r="H151" t="n">
         <v>1</v>
       </c>
-      <c r="I151" t="inlineStr">
+      <c r="I151" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102602023_nachlaufende_Kosten.xlsx</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>w4102602023 nachlaufende kosten ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5842,9 +6615,14 @@
       <c r="H152" t="n">
         <v>388</v>
       </c>
-      <c r="I152" t="inlineStr">
+      <c r="I152" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604411_Vertrieb_Region_Ost.xlsx</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>w4102604411 vertrieb region ost ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5872,9 +6650,14 @@
       <c r="H153" t="n">
         <v>26</v>
       </c>
-      <c r="I153" t="inlineStr">
+      <c r="I153" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604414_Halle_Boxberg.xlsx</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>w4102604414 halle boxberg ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5902,9 +6685,14 @@
       <c r="H154" t="n">
         <v>0</v>
       </c>
-      <c r="I154" t="inlineStr">
+      <c r="I154" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604501_Gehalt_BL_Region_Sued.xlsx</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>w4102604501 gehalt bl region sued ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5932,9 +6720,14 @@
       <c r="H155" t="n">
         <v>138</v>
       </c>
-      <c r="I155" t="inlineStr">
+      <c r="I155" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604611_Lager_Regon_Sued.xlsx</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>w4102604611 lager regon sued ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5962,9 +6755,14 @@
       <c r="H156" t="n">
         <v>34</v>
       </c>
-      <c r="I156" t="inlineStr">
+      <c r="I156" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604612_Recyclingplatz_Boxberg.xlsx</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>w4102604612 recyclingplatz boxberg ost aktiv</t>
         </is>
       </c>
     </row>
@@ -5992,9 +6790,14 @@
       <c r="H157" t="n">
         <v>0</v>
       </c>
-      <c r="I157" t="inlineStr">
+      <c r="I157" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604613_Basis_HR.xlsx</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>w4102604613 basis hr ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6022,9 +6825,14 @@
       <c r="H158" t="n">
         <v>42</v>
       </c>
-      <c r="I158" t="inlineStr">
+      <c r="I158" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604938_CB-AA_501_Spindler.xlsx</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>w4102604938 cb-aa 501 spindler ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6052,9 +6860,14 @@
       <c r="H159" t="n">
         <v>37</v>
       </c>
-      <c r="I159" t="inlineStr">
+      <c r="I159" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604940_CB-VT_475_Heilmann.xlsx</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>w4102604940 cb-vt 475 heilmann ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6082,9 +6895,14 @@
       <c r="H160" t="n">
         <v>47</v>
       </c>
-      <c r="I160" t="inlineStr">
+      <c r="I160" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604941_CB-TV_22E_Tayron_Hr_Lorenz.xlsx</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>w4102604941 cb-tv 22e tayron hr lorenz ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6112,9 +6930,14 @@
       <c r="H161" t="n">
         <v>30</v>
       </c>
-      <c r="I161" t="inlineStr">
+      <c r="I161" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604949_CB_-_VT_686_Passat_Fr_Kolber.xlsx</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>w4102604949 cb - vt 686 passat fr. kolber ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6142,9 +6965,14 @@
       <c r="H162" t="n">
         <v>35</v>
       </c>
-      <c r="I162" t="inlineStr">
+      <c r="I162" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604950_CB-TV_97_Hr_Mühlberg.xlsx</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>w4102604950 cb-tv 97 hr. mühlberg ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6172,9 +7000,14 @@
       <c r="H163" t="n">
         <v>7</v>
       </c>
-      <c r="I163" t="inlineStr">
+      <c r="I163" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102604951_PKW_Herr_Tymczy.xlsx</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>w4102604951 pkw herr tymczy ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6202,9 +7035,14 @@
       <c r="H164" t="n">
         <v>28</v>
       </c>
-      <c r="I164" t="inlineStr">
+      <c r="I164" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102607081_Abbr_Lager_radioakt_Abfälle_Los_3_EWN.xlsx</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>w4102607081 abbr.lager  radioakt. abfälle  los 3/ewn ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6232,9 +7070,14 @@
       <c r="H165" t="n">
         <v>7</v>
       </c>
-      <c r="I165" t="inlineStr">
+      <c r="I165" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102608246_RB_Kohlebunker_Brücke_Lübbenau.xlsx</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>w4102608246 rb kohlebunker/brücke lübbenau ost aktiv</t>
         </is>
       </c>
     </row>
@@ -6262,9 +7105,14 @@
       <c r="H166" t="n">
         <v>35</v>
       </c>
-      <c r="I166" t="inlineStr">
+      <c r="I166" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102651216_Bagger_CAT_326_07_FLN.xlsx</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>w4102651216 bagger cat 326 07 fln berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6292,9 +7140,14 @@
       <c r="H167" t="n">
         <v>7</v>
       </c>
-      <c r="I167" t="inlineStr">
+      <c r="I167" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102652709_CB-TV_96_Remault_Kangoo.xlsx</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>w4102652709 cb-tv 96 remault kangoo berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6322,9 +7175,14 @@
       <c r="H168" t="n">
         <v>232</v>
       </c>
-      <c r="I168" t="inlineStr">
+      <c r="I168" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102654411_VVK_Berlin.xlsx</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>w4102654411 vvk berlin berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6352,9 +7210,14 @@
       <c r="H169" t="n">
         <v>127</v>
       </c>
-      <c r="I169" t="inlineStr">
+      <c r="I169" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102654611_Lager_Region_Berlin.xlsx</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>w4102654611 lager region berlin berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6382,9 +7245,14 @@
       <c r="H170" t="n">
         <v>52</v>
       </c>
-      <c r="I170" t="inlineStr">
+      <c r="I170" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102654945_CB-_TV_300E_Hr_Kemper_Mercedes.xlsx</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>w4102654945 cb- tv 300e hr. kemper mercedes berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6412,9 +7280,14 @@
       <c r="H171" t="n">
         <v>40</v>
       </c>
-      <c r="I171" t="inlineStr">
+      <c r="I171" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102654946_CB-TV_65_Hr_Braun.xlsx</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>w4102654946 cb-tv 65 hr braun berlin aktiv</t>
         </is>
       </c>
     </row>
@@ -6442,13 +7315,189 @@
       <c r="H172" t="n">
         <v>27</v>
       </c>
-      <c r="I172" t="inlineStr">
+      <c r="I172" s="5" t="inlineStr">
         <is>
           <t>Projekt_W4102654947_CB-TV_200_Hr_Adil.xlsx</t>
         </is>
       </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>w4102654947 cb-tv 200 hr. adil berlin aktiv</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:J172"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I66" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I67" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I68" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I69" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I70" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I71" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I72" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I73" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I74" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I75" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I76" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I77" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I78" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I79" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I80" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I81" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I82" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I83" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I84" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I85" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I86" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I87" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I88" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I89" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I90" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I91" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I92" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I93" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I94" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I95" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I96" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I97" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I98" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I99" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I100" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I101" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I102" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I103" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I104" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I105" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I106" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I107" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I108" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I109" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I110" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I111" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I112" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I113" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I114" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I115" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I116" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I117" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I118" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I119" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I120" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I121" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I122" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I123" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I124" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I125" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I126" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I127" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I128" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I129" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I130" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I131" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I132" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I133" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I134" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I135" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I136" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I137" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I138" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I139" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I140" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I141" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I142" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I143" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I144" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I145" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I146" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I147" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I148" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I149" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I150" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I151" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I152" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I153" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I154" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I155" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I156" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I157" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I158" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I159" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I160" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I161" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I162" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I163" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I164" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I165" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I166" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I167" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I168" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I169" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I170" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I171" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I172" r:id="rId168"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>